<commit_message>
Align repository to QA Defect Lifecycle (1 Open, 2 Resolved defects)
</commit_message>
<xml_diff>
--- a/06-Test-Execution/API_Execution_Report.xlsx
+++ b/06-Test-Execution/API_Execution_Report.xlsx
@@ -1564,7 +1564,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>DEF-API-02</t>
+          <t>DEF-API-02 (Closed)</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>DEF-API-03</t>
+          <t>DEF-API-03 (Closed)</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">

</xml_diff>